<commit_message>
AI Agent:summarizer using Langgraph and few additonal changes
</commit_message>
<xml_diff>
--- a/learning/Complete_AI_Learning_Plan_With_Projects_and_Resources.xlsx
+++ b/learning/Complete_AI_Learning_Plan_With_Projects_and_Resources.xlsx
@@ -5,28 +5,42 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amanpatial/Desktop/Gen AI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amanpatial/Documents/projects/gen-ai-app/learning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3369AB-D3FC-4C43-88F1-0046B1A28A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166CAC93-8FC6-1743-B0C8-A8C6057C2927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MS Copilot" sheetId="4" r:id="rId1"/>
     <sheet name="Open Source" sheetId="1" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
     <sheet name="Tools " sheetId="3" r:id="rId4"/>
+    <sheet name="AWS" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MS Copilot'!$B$3:$D$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MS Copilot'!$B$3:$E$49</definedName>
   </definedNames>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="478">
   <si>
     <t>Day</t>
   </si>
@@ -1273,9 +1287,6 @@
     <t>Bonus (Advanced Developers)</t>
   </si>
   <si>
-    <t>Using Azure Functions, Logic Apps</t>
-  </si>
-  <si>
     <t>Power Virtual Agent SDK / APIs</t>
   </si>
   <si>
@@ -1285,9 +1296,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Creating and managing topics (trigger phrases, node structure, adoption card)</t>
-  </si>
-  <si>
     <t>Done</t>
   </si>
   <si>
@@ -1331,13 +1339,254 @@
   </si>
   <si>
     <t xml:space="preserve">MS Intra/AD Authentication integration with Agent and all possible options </t>
+  </si>
+  <si>
+    <t>Web Site as Knowledge source such as public site with F&amp;Q and Standard Open/Close Time</t>
+  </si>
+  <si>
+    <t>Web Site as Knowledge source such as Dataverse for structure database</t>
+  </si>
+  <si>
+    <t>Creating and managing topics (Adaptive card)</t>
+  </si>
+  <si>
+    <t>Using Azure Functions, Logic Apps, Azure AI Search, Azure SQL</t>
+  </si>
+  <si>
+    <t>n8n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Framework </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topics - Custom and Systems </t>
+  </si>
+  <si>
+    <t>Creating &amp; managing topics (Trigger phrases, Node structure, Adaptive Cards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power Fx function overview, solution fitment scenarios and MS power apps function guide </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Management - Set variable value,  System and custom environment variable   </t>
+  </si>
+  <si>
+    <t>Outcome Learning Notes</t>
+  </si>
+  <si>
+    <t>make.powerapps.com --&gt; tables</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A Tenant ID is a unique identifier for an organization within a cloud service, like Microsoft Entra ID (formerly Azure Active Directory). Within a single tenant ID for agent bot deployment in Power Platform, multiple environments can exist. A default environment is automatically created, but you can create additional environments like production or trial environments as needed. You can create new environments (e.g., trial or production) through the Power Platform admin center using the same tenant ID as your Copilot Studio e..g </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Power Platform admin center --&gt; environment</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Each environment is created under a Microsoft Entra tenant, and its resources can only be accessed by users within that tenant based on geo location.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Tenant id &lt;-1:!-&gt; Entra ID -1:N-&gt; Environement(S). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>All environments (except developer) can be managed via the Power Platform Admin Center. Developer env is managed by  Power Apps Developer Plan. Environments have two built-in roles - The Environment Admin, The Environment Maker</t>
+    </r>
+  </si>
+  <si>
+    <t>Copilot action - Flow try catch handling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Bedrock Agent Core </t>
+  </si>
+  <si>
+    <t>AWS IDE KIRO</t>
+  </si>
+  <si>
+    <t>AWS S3 Vector DB Support</t>
+  </si>
+  <si>
+    <t>AWS S3 BedRock Overview</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No authentication (Demo web site/ custom website with an iframe)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> provide embedded credentials or connection strings, but</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 'Authentication with Microsoft' (Teams, Power Apps, and Microsoft 365 Copilot )</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'Authentication manually' (Direct Line)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> providing the connection string only and config it using connection or traditional parameters configuration method.  In 'Authentication with Microsoft', The agent automatically uses Microsoft Entra ID authentication for Teams, Power Apps, and Microsoft 365 Copilot without requiring any manual setup. and uses 'Authentication manually'  for other channels such as mobile app.</t>
+    </r>
+  </si>
+  <si>
+    <t>Copilot action - integration with Share point file reading the excel sheet and print count</t>
+  </si>
+  <si>
+    <t>Authentication integration with Agent and all possible options overview</t>
+  </si>
+  <si>
+    <t>Configured 'Authentication manually' (Direct Line) using Dummy bot/agent and client id &amp; secret key from App created in KSG Student tenant Azure AD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User authentication using Copilot Studio Bot &amp; Flutter Native App integration over Direct Line API </t>
+  </si>
+  <si>
+    <t>Copilot Studio Agent &amp; Flutter Native App integration over Direct Line Channel/API</t>
+  </si>
+  <si>
+    <t>Amazon Q</t>
+  </si>
+  <si>
+    <t>Amazon Nova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event Type, Intent, Activity Channel, Channel Data learning </t>
+  </si>
+  <si>
+    <t>Channel and Token Forward Technique and extracation on bot server</t>
+  </si>
+  <si>
+    <t>Mobile app using flutter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress </t>
+  </si>
+  <si>
+    <t>Emergent - Vibe coding</t>
+  </si>
+  <si>
+    <t>Google NotebookLM</t>
+  </si>
+  <si>
+    <t>Hugging Face</t>
+  </si>
+  <si>
+    <t>Cursor IDE</t>
+  </si>
+  <si>
+    <t>WindSurf IDE</t>
+  </si>
+  <si>
+    <t>Olamma</t>
+  </si>
+  <si>
+    <t>OpenAI GPT-OSS</t>
+  </si>
+  <si>
+    <t>Databricks</t>
+  </si>
+  <si>
+    <t>FastAPI</t>
+  </si>
+  <si>
+    <t>Cohere</t>
+  </si>
+  <si>
+    <t>ReAct prompt framework</t>
+  </si>
+  <si>
+    <t>AWS SageMaker</t>
+  </si>
+  <si>
+    <t>AI UX prototyping</t>
+  </si>
+  <si>
+    <t>Figma/Canva/Miro/Gamma</t>
+  </si>
+  <si>
+    <t>Regex, Templates, ReAct/COT chains</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1367,8 +1616,23 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1381,8 +1645,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FFA3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1405,6 +1687,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1413,7 +1708,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1425,13 +1720,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1439,6 +1751,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF8FFA3"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1738,428 +2055,616 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2776CFE3-7CE5-034A-A49E-3430F643CD3A}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B2:D38"/>
+  <dimension ref="B2:E49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.1640625" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="68.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="1" max="1" width="2" customWidth="1"/>
+    <col min="2" max="2" width="32.1640625" customWidth="1"/>
+    <col min="3" max="3" width="76.1640625" customWidth="1"/>
+    <col min="4" max="4" width="27.1640625" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B2" s="9" t="s">
-        <v>429</v>
-      </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
         <v>385</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
+      <c r="D3" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
         <v>387</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="152" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C5" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>445</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="145" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
         <v>387</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
+        <v>453</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>387</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>454</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>455</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>454</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B9" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B10" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B11" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D15" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B8" s="5" t="s">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B18" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="5" t="s">
+      <c r="C18" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="C19" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="10" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B11" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B12" s="5" t="s">
+    <row r="21" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="5" t="s">
         <v>393</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>427</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B16" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="5" t="s">
-        <v>400</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>432</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" t="s">
+        <v>460</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B26" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B27" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B29" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B31" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>402</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B33" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B39" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B40" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B41" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B42" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B43" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B44" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="C44" s="6" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="22" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="23" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>402</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="25" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>405</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="26" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>406</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="29" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>410</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="30" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="5" t="s">
+      <c r="D44" s="6"/>
+      <c r="E44" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B45" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="5" t="s">
+      <c r="C45" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="D45" s="6"/>
+      <c r="E45" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B46" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="5" t="s">
+      <c r="C46" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B47" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4" ht="16" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="C35" s="6" t="s">
+      <c r="C47" s="5" t="s">
         <v>422</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="36" spans="2:4" ht="16" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>421</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="37" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>423</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="38" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>424</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>426</v>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B48" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="B49" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5" t="s">
+        <v>418</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:D38" xr:uid="{2776CFE3-7CE5-034A-A49E-3430F643CD3A}">
-    <filterColumn colId="2">
+  <autoFilter ref="B3:E49" xr:uid="{2776CFE3-7CE5-034A-A49E-3430F643CD3A}">
+    <filterColumn colId="3">
       <filters>
-        <filter val="In Progress"/>
+        <filter val="Not Started"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <mergeCells count="1">
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3794,11 +4299,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91FEDA53-78E6-8D42-BFC9-16515C26D988}">
-  <dimension ref="B2:E28"/>
+  <dimension ref="B2:E42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.6640625" customWidth="1"/>
     <col min="4" max="4" width="58.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.33203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -3818,367 +4323,495 @@
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="5" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="5" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
+      <c r="B5" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="15" t="s">
         <v>306</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="5" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
+      <c r="B6" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="15" t="s">
         <v>309</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="5" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
+      <c r="B7" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="15" t="s">
         <v>312</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="5" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="15" t="s">
         <v>315</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>319</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>320</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>322</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
+      <c r="B12" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="5" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="5" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="5" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="5" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="5" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="5" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="5" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="5" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="5" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="5" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="5" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="16" t="s">
         <v>366</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="5" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="16" t="s">
         <v>369</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="5" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B25" t="s">
+      <c r="B25" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="16" t="s">
         <v>372</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="5" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="16" t="s">
         <v>375</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="5" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B27" t="s">
+      <c r="B27" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="16" t="s">
         <v>378</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="5" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B28" t="s">
+      <c r="B28" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="16" t="s">
         <v>381</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="5" t="s">
         <v>382</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B29" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>465</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B30" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>383</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B31" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>437</v>
+      </c>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>463</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B33" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>464</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>466</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>467</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B36" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B37" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>469</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B38" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B39" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C40" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C41" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" t="s">
+        <v>477</v>
       </c>
     </row>
   </sheetData>
@@ -4196,15 +4829,93 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2375A9F0-676C-EE49-ADE9-0C77AE02FD61}">
-  <dimension ref="D4"/>
+  <dimension ref="C4:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="28.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="30.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D4" t="s">
+    <row r="4" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C4" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>383</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C5" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D6" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D7" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>475</v>
+      </c>
+      <c r="D9" t="s">
+        <v>476</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7531EC7-7F0E-BF44-B715-B2D3E9B7C7F7}">
+  <dimension ref="F3:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="45.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="4" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="5" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="6" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="7" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="8" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F8" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="9" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F9" t="s">
+        <v>474</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add evals test criteria and grader code
</commit_message>
<xml_diff>
--- a/learning/Complete_AI_Learning_Plan_With_Projects_and_Resources.xlsx
+++ b/learning/Complete_AI_Learning_Plan_With_Projects_and_Resources.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11102"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amanpatial/Documents/projects/gen-ai-app/learning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166CAC93-8FC6-1743-B0C8-A8C6057C2927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F862D9CD-BA3D-2945-BD3E-F870855928F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,8 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
     <sheet name="Tools " sheetId="3" r:id="rId4"/>
     <sheet name="AWS" sheetId="5" r:id="rId5"/>
+    <sheet name="Gen AI Stack" sheetId="6" r:id="rId6"/>
+    <sheet name="Developer" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MS Copilot'!$B$3:$E$49</definedName>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="654">
   <si>
     <t>Day</t>
   </si>
@@ -1581,14 +1583,810 @@
   <si>
     <t>Regex, Templates, ReAct/COT chains</t>
   </si>
+  <si>
+    <t>GenAI + Agentic AI Platform Comparison (Google Cloud vs Microsoft Azure vs AWS Open Source)</t>
+  </si>
+  <si>
+    <t>Models &amp; Core GenAI</t>
+  </si>
+  <si>
+    <t>Capability</t>
+  </si>
+  <si>
+    <t>Google Cloud</t>
+  </si>
+  <si>
+    <t>Microsoft Azure</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>Flagship LLMs</t>
+  </si>
+  <si>
+    <t>Gemini 1.5 / 2.x</t>
+  </si>
+  <si>
+    <t>GPT-4 / 4.1 / GPT-5</t>
+  </si>
+  <si>
+    <t>Claude, Llama, Titan</t>
+  </si>
+  <si>
+    <t>LLM Access Layer</t>
+  </si>
+  <si>
+    <t>Vertex AI / Gemini API</t>
+  </si>
+  <si>
+    <t>Azure OpenAI Service</t>
+  </si>
+  <si>
+    <t>Amazon Bedrock</t>
+  </si>
+  <si>
+    <t>Multimodal Support</t>
+  </si>
+  <si>
+    <t>Native (text, image, video, long context)</t>
+  </si>
+  <si>
+    <t>Strong (Vision, Image, Video via OpenAI)</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t>Context Window</t>
+  </si>
+  <si>
+    <t>Up to 1M+ tokens</t>
+  </si>
+  <si>
+    <t>~128k tokens</t>
+  </si>
+  <si>
+    <t>~200k tokens (Claude)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category </t>
+  </si>
+  <si>
+    <t>Native Agent SDK</t>
+  </si>
+  <si>
+    <t>Google ADK</t>
+  </si>
+  <si>
+    <t>AutoGen, Semantic Kernel</t>
+  </si>
+  <si>
+    <t>Bedrock Agent SDK</t>
+  </si>
+  <si>
+    <t>Open-Source Agent Frameworks</t>
+  </si>
+  <si>
+    <t>Agent Orchestration Style</t>
+  </si>
+  <si>
+    <t>Tool-driven</t>
+  </si>
+  <si>
+    <t>Multi-agent &amp; planner-driven</t>
+  </si>
+  <si>
+    <t>Task-driven</t>
+  </si>
+  <si>
+    <t>Stateful / Graph-based Agents</t>
+  </si>
+  <si>
+    <t>Via LangGraph</t>
+  </si>
+  <si>
+    <t>Strong via LangGraph + AutoGen</t>
+  </si>
+  <si>
+    <t>Primary Use</t>
+  </si>
+  <si>
+    <t>App-centric agents</t>
+  </si>
+  <si>
+    <t>Enterprise copilots</t>
+  </si>
+  <si>
+    <t>Controlled workflows</t>
+  </si>
+  <si>
+    <t>Agentic AI – SDKs, Frameworks</t>
+  </si>
+  <si>
+    <t>Agent Platform</t>
+  </si>
+  <si>
+    <t>Vertex AI</t>
+  </si>
+  <si>
+    <t>Microsoft AI Foundry</t>
+  </si>
+  <si>
+    <t>Build, deploy, scale GenAI apps</t>
+  </si>
+  <si>
+    <t>Lifecycle, governance &amp; orchestration</t>
+  </si>
+  <si>
+    <t>Model &amp; agent hosting</t>
+  </si>
+  <si>
+    <t>Tool / Action Execution</t>
+  </si>
+  <si>
+    <t>Vertex Extensions</t>
+  </si>
+  <si>
+    <t>Graph API, Functions</t>
+  </si>
+  <si>
+    <t>Lambda</t>
+  </si>
+  <si>
+    <t>Agent Lifecycle Mgmt</t>
+  </si>
+  <si>
+    <t>End-to-end</t>
+  </si>
+  <si>
+    <t>Limited</t>
+  </si>
+  <si>
+    <t>Agent Platform &amp; Control Plane</t>
+  </si>
+  <si>
+    <t>Native Vector DB</t>
+  </si>
+  <si>
+    <t>Vertex Vector Search</t>
+  </si>
+  <si>
+    <t>Azure AI Search (vector)</t>
+  </si>
+  <si>
+    <t>OpenSearch / pgvector</t>
+  </si>
+  <si>
+    <t>Open-Source RAG Framework</t>
+  </si>
+  <si>
+    <t>LlamaIndex, LangChain</t>
+  </si>
+  <si>
+    <t>Enterprise Search</t>
+  </si>
+  <si>
+    <t>Vertex AI Search</t>
+  </si>
+  <si>
+    <t>Azure Cognitive Search</t>
+  </si>
+  <si>
+    <t>Amazon Kendra</t>
+  </si>
+  <si>
+    <t>Memory Strategy</t>
+  </si>
+  <si>
+    <t>Vector DB + OS memory</t>
+  </si>
+  <si>
+    <t>Built-in + OS memory</t>
+  </si>
+  <si>
+    <t>DIY</t>
+  </si>
+  <si>
+    <t>RAG, Memory &amp; Knowledge (with LlamaIndex)</t>
+  </si>
+  <si>
+    <t>Primary SDKs</t>
+  </si>
+  <si>
+    <t>Python, Java, Node.js, Go</t>
+  </si>
+  <si>
+    <t>Python, C#, Java, JS</t>
+  </si>
+  <si>
+    <t>Python, Java, JS</t>
+  </si>
+  <si>
+    <t>GenAI SDKs</t>
+  </si>
+  <si>
+    <t>Gemini API, Vertex SDK</t>
+  </si>
+  <si>
+    <t>Azure OpenAI SDK</t>
+  </si>
+  <si>
+    <t>Bedrock SDK</t>
+  </si>
+  <si>
+    <t>IDE / Coding AI</t>
+  </si>
+  <si>
+    <t>Gemini Code Assist</t>
+  </si>
+  <si>
+    <t>GitHub Copilot</t>
+  </si>
+  <si>
+    <t>CodeWhisperer</t>
+  </si>
+  <si>
+    <t>Developer Experience &amp; SDKs</t>
+  </si>
+  <si>
+    <t>ML Frameworks</t>
+  </si>
+  <si>
+    <t>TensorFlow, JAX, Keras</t>
+  </si>
+  <si>
+    <t>PyTorch</t>
+  </si>
+  <si>
+    <t>Workflow Orchestration</t>
+  </si>
+  <si>
+    <t>Vertex Pipelines</t>
+  </si>
+  <si>
+    <t>Azure ML Pipelines</t>
+  </si>
+  <si>
+    <t>Step Functions</t>
+  </si>
+  <si>
+    <t>Agent Workflow (OS)</t>
+  </si>
+  <si>
+    <t>LangGraph</t>
+  </si>
+  <si>
+    <t>Analytics + AI</t>
+  </si>
+  <si>
+    <t>BigQuery ML</t>
+  </si>
+  <si>
+    <t>Fabric / Synapse</t>
+  </si>
+  <si>
+    <t>Redshift / Athena</t>
+  </si>
+  <si>
+    <t>ML, Workflow &amp; Data Integration</t>
+  </si>
+  <si>
+    <t>Responsible AI</t>
+  </si>
+  <si>
+    <t>Strong</t>
+  </si>
+  <si>
+    <t>Best-in-class</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>Identity &amp; Access</t>
+  </si>
+  <si>
+    <t>IAM, VPC-SC</t>
+  </si>
+  <si>
+    <t>Entra ID, RBAC</t>
+  </si>
+  <si>
+    <t>IAM</t>
+  </si>
+  <si>
+    <t>Monitoring &amp; Eval</t>
+  </si>
+  <si>
+    <t>Vertex Monitoring</t>
+  </si>
+  <si>
+    <t>AI Foundry + Azure Monitor</t>
+  </si>
+  <si>
+    <t>CloudWatch</t>
+  </si>
+  <si>
+    <t>Enterprise Readiness</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Very High</t>
+  </si>
+  <si>
+    <t>Governance, Security &amp; Responsible AI</t>
+  </si>
+  <si>
+    <t>Google ADK is a developer toolkit for building agents, whereas Microsoft AI Foundry is an enterprise platform for running and governing agentic systems at scale.</t>
+  </si>
+  <si>
+    <t>Cloud-Native</t>
+  </si>
+  <si>
+    <t>Open-Source Alternative</t>
+  </si>
+  <si>
+    <t>Google: Python, Java, Node.js, GoAzure: Python, C#, Java, JSAWS: Python, Java, JS</t>
+  </si>
+  <si>
+    <t>GenAI / LLM SDKs</t>
+  </si>
+  <si>
+    <t>Google: Gemini API, Vertex SDKAzure: Azure OpenAI SDKAWS: Bedrock SDK</t>
+  </si>
+  <si>
+    <t>Google ADK, AutoGen, Bedrock Agents</t>
+  </si>
+  <si>
+    <t>Gemini Code Assist, GitHub Copilot, CodeWhisperer</t>
+  </si>
+  <si>
+    <t>Low-Code / Studio</t>
+  </si>
+  <si>
+    <t>Vertex AI Studio, Azure AI Studio, Bedrock Console</t>
+  </si>
+  <si>
+    <t>Workflow / Agent Orchestration</t>
+  </si>
+  <si>
+    <t>Vertex Pipelines, Azure ML Pipelines, Step Functions</t>
+  </si>
+  <si>
+    <t>RAG / Memory Integration</t>
+  </si>
+  <si>
+    <t>Vertex Vector Search, Azure AI Search, OpenSearch</t>
+  </si>
+  <si>
+    <r>
+      <t>Hugging Face Transformers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Python/JS), OpenAI Python SDK (cross-cloud), LangChain SDKs</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Hugging Face Hub</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, OpenLLM, LangChain, LlamaIndex</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>LangChain</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, LangGraph, AutoGPT, OpenAssistant</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CodeGeeX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, CodeGen, PolyCoder</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Gradio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Streamlit, Jupyter + LangChain UI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Prefect</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Airflow, LangGraph, Dagster</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Chroma</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Weaviate, FAISS, LlamaIndex</t>
+    </r>
+  </si>
+  <si>
+    <t>Developer Experience &amp; SDKs — Open-Source Alternatives</t>
+  </si>
+  <si>
+    <r>
+      <t>Cloud-native SDKs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> are enterprise-ready, secure, and integrated with governance, monitoring, and compliance.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Open-source SDKs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (LangChain, LangGraph, LlamaIndex, Hugging Face, etc.) are </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>cross-cloud, highly customizable, and research-friendly</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Often, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>hybrid approach</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is used: open-source for experimentation + cloud-native for production deployment.</t>
+    </r>
+  </si>
+  <si>
+    <t>Open-Source Alternatives</t>
+  </si>
+  <si>
+    <t>Evaluation Tools</t>
+  </si>
+  <si>
+    <t>Vertex AI Evaluations, Model Card Toolkit</t>
+  </si>
+  <si>
+    <t>Responsible AI Dashboard, Model Insights</t>
+  </si>
+  <si>
+    <t>SageMaker Clarify, Model Monitor</t>
+  </si>
+  <si>
+    <r>
+      <t>OpenAI Evals</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LangChain Evaluator</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HydraEval</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PromptBench</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LM-Eval-Harness</t>
+    </r>
+  </si>
+  <si>
+    <t>Bias, fairness, performance, safety</t>
+  </si>
+  <si>
+    <t>Bias, fairness, explainability</t>
+  </si>
+  <si>
+    <t>Bias, fairness, production monitoring</t>
+  </si>
+  <si>
+    <t>Benchmarking, prompt evaluation, alignment, RAG QA testing</t>
+  </si>
+  <si>
+    <t>Evaluation / Model Assessment Tools</t>
+  </si>
+  <si>
+    <t>Cloud-native evaluation tools handle governance and production monitoring, while open-source frameworks like LangChain Evaluator, LlamaIndex, and OpenAI Evals enable flexible benchmarking and alignment testing across platforms</t>
+  </si>
+  <si>
+    <t>MPT, Falcon, LLaMA, OpenLLaMA, Vicuna, OpenAssistant</t>
+  </si>
+  <si>
+    <t>Hugging Face Transformers, OpenLLM, text-generation-webui</t>
+  </si>
+  <si>
+    <t>OpenFlamingo, BLIP-2, MiniGPT-4, OpenDALL·E</t>
+  </si>
+  <si>
+    <t>Varies by model (e.g., 2k–128k tokens in LLaMA 3 / MPT-30B)</t>
+  </si>
+  <si>
+    <t>LangChain, LangGraph, AutoGPT, OpenAssistant, SuperAGI</t>
+  </si>
+  <si>
+    <t>LangChain Agents, LangGraph, AutoGPT workflow</t>
+  </si>
+  <si>
+    <t>LangGraph, AutoGPT, BabyAGI</t>
+  </si>
+  <si>
+    <t>Experimentation, research, RAG agents, multi-tool agents</t>
+  </si>
+  <si>
+    <r>
+      <t>LocalStack + LangChain / LangGraph</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Custom Docker + Hugging Face Inference</t>
+    </r>
+  </si>
+  <si>
+    <t>Developer experimentation, self-hosted agents</t>
+  </si>
+  <si>
+    <t>LangChain Tools, OpenAssistant tool integration</t>
+  </si>
+  <si>
+    <t>LangGraph + Prefect / Airflow orchestration</t>
+  </si>
+  <si>
+    <t>FAISS, Chroma, Weaviate, Milvus, Pinecone (self-hosted)</t>
+  </si>
+  <si>
+    <t>LlamaIndex, LangChain, Haystack, OpenRAG</t>
+  </si>
+  <si>
+    <t>Weaviate, Milvus + Haystack</t>
+  </si>
+  <si>
+    <t>LangChain memory modules, Chroma / FAISS embedding storage</t>
+  </si>
+  <si>
+    <t>Hugging Face Transformers, OpenLLM, LangChain SDK</t>
+  </si>
+  <si>
+    <t>OpenAI Python SDK, Hugging Face Hub SDK, text-generation-webui</t>
+  </si>
+  <si>
+    <t>CodeGeeX, CodeGen, PolyCoder, CodeT5</t>
+  </si>
+  <si>
+    <t>PyTorch, TensorFlow, JAX, Flax, Hugging Face Accelerate</t>
+  </si>
+  <si>
+    <t>Prefect, Airflow, Dagster, Kedro</t>
+  </si>
+  <si>
+    <t>DuckDB, Polars, Pandas + Hugging Face embeddings</t>
+  </si>
+  <si>
+    <t>Eval frameworks: OpenAI Evals, HydraEval, LM-Eval-Harness</t>
+  </si>
+  <si>
+    <t>Keycloak, Ory Kratos / Ory Keto</t>
+  </si>
+  <si>
+    <t>Prometheus + Grafana + custom eval scripts</t>
+  </si>
+  <si>
+    <t>Varies by deployment; suitable for dev/test</t>
+  </si>
+  <si>
+    <t>Open-source frameworks like LangChain, LangGraph, and LlamaIndex complement cloud-native platforms by enabling flexible agentic workflows, RAG pipelines, and evaluation, while cloud-native tools provide governance, scale, and enterprise readiness.”</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1631,8 +2429,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1660,6 +2473,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FFA3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1703,28 +2522,28 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1735,15 +2554,46 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2066,12 +2916,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="20" t="s">
         <v>427</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
@@ -2127,7 +2977,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:5" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>387</v>
       </c>
@@ -2141,7 +2991,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="48" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:5" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
         <v>387</v>
       </c>
@@ -4326,7 +5176,7 @@
       <c r="B3" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="14" t="s">
         <v>299</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -4340,7 +5190,7 @@
       <c r="B4" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="14" t="s">
         <v>302</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -4354,7 +5204,7 @@
       <c r="B5" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>306</v>
       </c>
       <c r="D5" s="5" t="s">
@@ -4368,7 +5218,7 @@
       <c r="B6" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="14" t="s">
         <v>309</v>
       </c>
       <c r="D6" s="5" t="s">
@@ -4382,7 +5232,7 @@
       <c r="B7" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="14" t="s">
         <v>312</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -4396,7 +5246,7 @@
       <c r="B8" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="14" t="s">
         <v>315</v>
       </c>
       <c r="D8" s="5" t="s">
@@ -4609,7 +5459,7 @@
       <c r="C23" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D23" s="15" t="s">
         <v>366</v>
       </c>
       <c r="E23" s="5" t="s">
@@ -4623,7 +5473,7 @@
       <c r="C24" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="D24" s="16" t="s">
+      <c r="D24" s="15" t="s">
         <v>369</v>
       </c>
       <c r="E24" s="5" t="s">
@@ -4637,7 +5487,7 @@
       <c r="C25" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="D25" s="15" t="s">
         <v>372</v>
       </c>
       <c r="E25" s="5" t="s">
@@ -4651,7 +5501,7 @@
       <c r="C26" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="D26" s="16" t="s">
+      <c r="D26" s="15" t="s">
         <v>375</v>
       </c>
       <c r="E26" s="5" t="s">
@@ -4665,7 +5515,7 @@
       <c r="C27" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="D27" s="16" t="s">
+      <c r="D27" s="15" t="s">
         <v>378</v>
       </c>
       <c r="E27" s="5" t="s">
@@ -4679,7 +5529,7 @@
       <c r="C28" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="15" t="s">
         <v>381</v>
       </c>
       <c r="E28" s="5" t="s">
@@ -4690,7 +5540,7 @@
       <c r="B29" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="16" t="s">
         <v>465</v>
       </c>
       <c r="D29" s="5"/>
@@ -4700,7 +5550,7 @@
       <c r="B30" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="17" t="s">
         <v>383</v>
       </c>
       <c r="D30" s="5"/>
@@ -4710,7 +5560,7 @@
       <c r="B31" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="17" t="s">
         <v>437</v>
       </c>
       <c r="D31" s="5"/>
@@ -4720,7 +5570,7 @@
       <c r="B32" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C32" s="19" t="s">
+      <c r="C32" s="18" t="s">
         <v>463</v>
       </c>
       <c r="D32" s="5"/>
@@ -4730,7 +5580,7 @@
       <c r="B33" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C33" s="20" t="s">
+      <c r="C33" s="19" t="s">
         <v>464</v>
       </c>
       <c r="D33" s="5"/>
@@ -4740,7 +5590,7 @@
       <c r="B34" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="14" t="s">
         <v>466</v>
       </c>
       <c r="D34" s="5"/>
@@ -4750,7 +5600,7 @@
       <c r="B35" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="14" t="s">
         <v>467</v>
       </c>
       <c r="D35" s="5"/>
@@ -4760,7 +5610,7 @@
       <c r="B36" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="C36" s="16" t="s">
         <v>468</v>
       </c>
       <c r="D36" s="5"/>
@@ -4770,7 +5620,7 @@
       <c r="B37" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="C37" s="16" t="s">
         <v>469</v>
       </c>
       <c r="D37" s="5"/>
@@ -4780,7 +5630,7 @@
       <c r="B38" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C38" s="17" t="s">
+      <c r="C38" s="16" t="s">
         <v>470</v>
       </c>
       <c r="D38" s="5"/>
@@ -4921,4 +5771,745 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18A0FE89-F433-864D-952A-3471FC3AE203}">
+  <dimension ref="A2:G36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.33203125" customWidth="1"/>
+    <col min="6" max="6" width="60.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" s="27" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="23" t="s">
+        <v>478</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="35"/>
+    </row>
+    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="36" t="s">
+        <v>500</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>480</v>
+      </c>
+      <c r="C3" s="37" t="s">
+        <v>481</v>
+      </c>
+      <c r="D3" s="37" t="s">
+        <v>482</v>
+      </c>
+      <c r="E3" s="37" t="s">
+        <v>483</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="22" t="s">
+        <v>479</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>485</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>486</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>487</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="22"/>
+      <c r="B5" s="25" t="s">
+        <v>488</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>489</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>490</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>491</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="22"/>
+      <c r="B6" s="25" t="s">
+        <v>492</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>493</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>494</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>495</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="22"/>
+      <c r="B7" s="25" t="s">
+        <v>496</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>497</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>498</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>499</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="22" t="s">
+        <v>517</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>501</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>502</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>503</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>504</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="22"/>
+      <c r="B9" s="28" t="s">
+        <v>506</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>507</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>508</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>509</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="22"/>
+      <c r="B10" s="28" t="s">
+        <v>510</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>511</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>512</v>
+      </c>
+      <c r="E10" s="30" t="s">
+        <v>511</v>
+      </c>
+      <c r="F10" s="30" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="22"/>
+      <c r="B11" s="28" t="s">
+        <v>513</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>514</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>515</v>
+      </c>
+      <c r="E11" s="30" t="s">
+        <v>516</v>
+      </c>
+      <c r="F11" s="30" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="22" t="s">
+        <v>531</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>518</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>519</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>520</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>491</v>
+      </c>
+      <c r="F12" s="26" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="22"/>
+      <c r="B13" s="25" t="s">
+        <v>297</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>521</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>522</v>
+      </c>
+      <c r="E13" s="31" t="s">
+        <v>523</v>
+      </c>
+      <c r="F13" s="31" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="22"/>
+      <c r="B14" s="25" t="s">
+        <v>524</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>525</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>526</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>527</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="22"/>
+      <c r="B15" s="25" t="s">
+        <v>528</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>495</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>529</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>530</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="32" t="s">
+        <v>546</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>532</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>533</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>534</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>535</v>
+      </c>
+      <c r="F16" s="30" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="32"/>
+      <c r="B17" s="28" t="s">
+        <v>536</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>537</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>537</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>537</v>
+      </c>
+      <c r="F17" s="30" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="32"/>
+      <c r="B18" s="28" t="s">
+        <v>538</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>539</v>
+      </c>
+      <c r="D18" s="30" t="s">
+        <v>540</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>541</v>
+      </c>
+      <c r="F18" s="30" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="32"/>
+      <c r="B19" s="28" t="s">
+        <v>542</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>543</v>
+      </c>
+      <c r="D19" s="30" t="s">
+        <v>544</v>
+      </c>
+      <c r="E19" s="30" t="s">
+        <v>545</v>
+      </c>
+      <c r="F19" s="30" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="22" t="s">
+        <v>559</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>547</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>548</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>549</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>550</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="22"/>
+      <c r="B21" s="25" t="s">
+        <v>551</v>
+      </c>
+      <c r="C21" s="31" t="s">
+        <v>552</v>
+      </c>
+      <c r="D21" s="31" t="s">
+        <v>553</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>554</v>
+      </c>
+      <c r="F21" s="31" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="22"/>
+      <c r="B22" s="25" t="s">
+        <v>555</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>556</v>
+      </c>
+      <c r="D22" s="31" t="s">
+        <v>557</v>
+      </c>
+      <c r="E22" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>560</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>561</v>
+      </c>
+      <c r="D23" s="30" t="s">
+        <v>562</v>
+      </c>
+      <c r="E23" s="30" t="s">
+        <v>562</v>
+      </c>
+      <c r="F23" s="28" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="33"/>
+      <c r="B24" s="28" t="s">
+        <v>563</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>564</v>
+      </c>
+      <c r="D24" s="30" t="s">
+        <v>565</v>
+      </c>
+      <c r="E24" s="30" t="s">
+        <v>566</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="33"/>
+      <c r="B25" s="28" t="s">
+        <v>567</v>
+      </c>
+      <c r="C25" s="29" t="s">
+        <v>568</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>568</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>568</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="33"/>
+      <c r="B26" s="28" t="s">
+        <v>569</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>570</v>
+      </c>
+      <c r="D26" s="30" t="s">
+        <v>571</v>
+      </c>
+      <c r="E26" s="30" t="s">
+        <v>572</v>
+      </c>
+      <c r="F26" s="28" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="32" t="s">
+        <v>589</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>574</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>575</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>576</v>
+      </c>
+      <c r="E27" s="31" t="s">
+        <v>577</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="32"/>
+      <c r="B28" s="25" t="s">
+        <v>578</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>579</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>580</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>581</v>
+      </c>
+      <c r="F28" s="31" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="32"/>
+      <c r="B29" s="25" t="s">
+        <v>582</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>583</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>584</v>
+      </c>
+      <c r="E29" s="31" t="s">
+        <v>585</v>
+      </c>
+      <c r="F29" s="31" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="32"/>
+      <c r="B30" s="25" t="s">
+        <v>586</v>
+      </c>
+      <c r="C30" s="31" t="s">
+        <v>587</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>588</v>
+      </c>
+      <c r="E30" s="31" t="s">
+        <v>587</v>
+      </c>
+      <c r="F30" s="31" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="32" t="s">
+        <v>625</v>
+      </c>
+      <c r="B31" s="28" t="s">
+        <v>616</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>617</v>
+      </c>
+      <c r="D31" s="28" t="s">
+        <v>618</v>
+      </c>
+      <c r="E31" s="28" t="s">
+        <v>619</v>
+      </c>
+      <c r="F31" s="28" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="32"/>
+      <c r="B32" s="28" t="s">
+        <v>297</v>
+      </c>
+      <c r="C32" s="28" t="s">
+        <v>621</v>
+      </c>
+      <c r="D32" s="28" t="s">
+        <v>622</v>
+      </c>
+      <c r="E32" s="28" t="s">
+        <v>623</v>
+      </c>
+      <c r="F32" s="28" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>653</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BB9EF17-9BE6-D94D-960B-53230AEE4336}">
+  <dimension ref="F4:H17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="63.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="70.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F4" s="21" t="s">
+        <v>611</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+    </row>
+    <row r="5" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F5" s="34" t="s">
+        <v>385</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>591</v>
+      </c>
+      <c r="H5" s="34" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="6" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F6" s="34" t="s">
+        <v>547</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>593</v>
+      </c>
+      <c r="H6" s="24" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="7" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F7" s="34" t="s">
+        <v>594</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>595</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="8" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F8" s="34" t="s">
+        <v>505</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="9" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F9" s="34" t="s">
+        <v>555</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>597</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="10" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F10" s="34" t="s">
+        <v>598</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="11" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F11" s="34" t="s">
+        <v>600</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="12" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F12" s="34" t="s">
+        <v>602</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="15" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F15" s="9" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="16" spans="6:8" x14ac:dyDescent="0.2">
+      <c r="F16" s="9" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>614</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F4:H4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>